<commit_message>
QA: update test cases
</commit_message>
<xml_diff>
--- a/QA/test-cases-happy-path.xlsx
+++ b/QA/test-cases-happy-path.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://alixpartners-my.sharepoint.com/personal/alejandro_lupo_alixpartners_com/Documents/Desktop/Hackathon/QA/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://alixpartners-my.sharepoint.com/personal/alejandro_lupo_alixpartners_com/Documents/Desktop/Hackathon/AP.Hackathon.FE/QA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{39E71973-958D-481D-892D-BE847B12FA85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BA8EAAF0-94E7-4002-BEC1-2CDBA42AD727}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{91D0F871-20BF-4DDD-8E1D-16B684D0527F}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{D6094198-F97C-4B20-A169-48DBA0FE44A6}"/>
   </bookViews>
   <sheets>
     <sheet name="Happy Path" sheetId="1" r:id="rId1"/>
@@ -62,205 +62,205 @@
     <t>TC-001</t>
   </si>
   <si>
-    <t>Flujo 1 — Análisis de Dotación</t>
-  </si>
-  <si>
-    <t>Carga de archivo Excel válido</t>
+    <t>Flow 1 — Roster Analysis</t>
+  </si>
+  <si>
+    <t>Upload a valid Excel file</t>
   </si>
   <si>
     <t>WorkshopRoster.xlsx</t>
   </si>
   <si>
-    <t>El usuario tiene WorkshopRoster.xlsx disponible localmente</t>
-  </si>
-  <si>
-    <t>1. Navegar a la pantalla de Análisis de Dotación
-2. Seleccionar el modo Upload
-3. Arrastrar o seleccionar WorkshopRoster.xlsx
-4. Confirmar la carga</t>
-  </si>
-  <si>
-    <t>El archivo es aceptado. El sistema parsea las columnas, muestra el total de empleados correctamente y habilita la vista de análisis.</t>
+    <t>User has WorkshopRoster.xlsx available locally</t>
+  </si>
+  <si>
+    <t>1. Navigate to the Roster Analysis screen
+2. Select Upload mode
+3. Drag or select WorkshopRoster.xlsx
+4. Confirm the upload</t>
+  </si>
+  <si>
+    <t>File is accepted. System parses the columns, displays the correct total headcount and enables the analysis view.</t>
   </si>
   <si>
     <t>TC-002</t>
   </si>
   <si>
-    <t>Carga de dotación por pegado desde portapapeles</t>
-  </si>
-  <si>
-    <t>El usuario tiene los datos del roster copiados en el portapapeles desde una planilla (formato TSV)</t>
-  </si>
-  <si>
-    <t>1. Navegar a la pantalla de Análisis de Dotación
-2. Seleccionar el modo Paste
-3. Hacer clic en la zona de pegado
-4. Presionar Ctrl+V</t>
-  </si>
-  <si>
-    <t>El sistema detecta y mapea las columnas automáticamente. Se muestra una preview con las primeras 4 filas y la cantidad de filas/columnas detectadas. El usuario puede confirmar la carga.</t>
+    <t>Load roster by pasting from clipboard</t>
+  </si>
+  <si>
+    <t>User has roster data copied to the clipboard from a spreadsheet (TSV format)</t>
+  </si>
+  <si>
+    <t>1. Navigate to the Roster Analysis screen
+2. Select Paste mode
+3. Click the paste area
+4. Press Ctrl+V</t>
+  </si>
+  <si>
+    <t>System auto-detects and maps columns. A preview table shows the first 4 rows and the detected row/column count. User can confirm the upload.</t>
   </si>
   <si>
     <t>TC-003</t>
   </si>
   <si>
-    <t>KPIs de dotación: headcount y costos</t>
-  </si>
-  <si>
-    <t>TC-001 o TC-002 aprobado</t>
-  </si>
-  <si>
-    <t>1. Observar la fila de KPIs en la pantalla de Análisis de Dotación</t>
-  </si>
-  <si>
-    <t>Se muestran: Total Headcount (total de filas), Total Labor Spend (suma de FLC), Avg Cost/Employee (Total Labor Spend / Headcount), Median Cost/Employee (mediana de FLC). Valores matemáticamente consistentes.</t>
+    <t>Roster KPIs: headcount and costs</t>
+  </si>
+  <si>
+    <t>TC-001 or TC-002 passed</t>
+  </si>
+  <si>
+    <t>1. Observe the KPI row on the Roster Analysis screen</t>
+  </si>
+  <si>
+    <t>Displayed correctly: Total Headcount (total rows in file), Total Labor Spend (sum of FLC), Avg Cost/Employee (Total Labor Spend / Headcount), Median Cost/Employee (median of FLC values). Values are mathematically consistent.</t>
   </si>
   <si>
     <t>TC-004</t>
   </si>
   <si>
-    <t>KPIs de dotación: senior ratio y concentración de costos</t>
-  </si>
-  <si>
-    <t>1. Observar la segunda fila de KPIs</t>
-  </si>
-  <si>
-    <t>Se muestran: Nº de Funciones (valores únicos de Job Function), Nº de Países (valores únicos de Country), Senior Ratio (% headcount VP o Director), Cost Concentration (% del gasto del top 25% de empleados por FLC). Valores consistentes con los datos.</t>
+    <t>Roster KPIs: senior ratio and cost concentration</t>
+  </si>
+  <si>
+    <t>1. Observe the second KPI row</t>
+  </si>
+  <si>
+    <t>Displayed: No. of Functions (unique Job Function values), No. of Countries (unique Country values), Senior Ratio (% headcount with Seniority = VP or Director), Cost Concentration (% of total spend from top 25% earners by FLC). Values consistent with file data.</t>
   </si>
   <si>
     <t>TC-005</t>
   </si>
   <si>
-    <t>Desglose de headcount por Job Function</t>
-  </si>
-  <si>
-    <t>1. Localizar el gráfico de barras Headcount by Function</t>
-  </si>
-  <si>
-    <t>Gráfico de barras horizontales ordenado de mayor a menor. Una barra por valor único en Job Function. La suma de todas las barras es igual al headcount total.</t>
+    <t>Headcount breakdown by Job Function</t>
+  </si>
+  <si>
+    <t>1. Locate the Headcount by Function bar chart</t>
+  </si>
+  <si>
+    <t>Horizontal bar chart sorted descending. One bar per unique Job Function value. Sum of all bars equals total headcount.</t>
   </si>
   <si>
     <t>TC-006</t>
   </si>
   <si>
-    <t>Desglose de headcount por Seniority</t>
-  </si>
-  <si>
-    <t>1. Localizar el gráfico Seniority Distribution</t>
-  </si>
-  <si>
-    <t>Gráfico de barras horizontales ordenado según la jerarquía organizacional (Executive → VP → Director → Manager → Staff). Una barra por nivel. La suma es igual al headcount total.</t>
+    <t>Headcount breakdown by Seniority</t>
+  </si>
+  <si>
+    <t>1. Locate the Seniority Distribution bar chart</t>
+  </si>
+  <si>
+    <t>Horizontal bar chart ordered by org hierarchy (Executive -&gt; VP -&gt; Director -&gt; Manager -&gt; Staff). One bar per level. Sum equals total headcount.</t>
   </si>
   <si>
     <t>TC-007</t>
   </si>
   <si>
-    <t>Desglose de gasto en personal por función</t>
-  </si>
-  <si>
-    <t>1. Localizar el gráfico Labor Spend by Function</t>
-  </si>
-  <si>
-    <t>Gráfico de barras horizontales con FLC total agrupado por Job Function. La suma de todas las barras es igual al Total Labor Spend del KPI.</t>
+    <t>Labor spend breakdown by function</t>
+  </si>
+  <si>
+    <t>1. Locate the Labor Spend by Function chart</t>
+  </si>
+  <si>
+    <t>Horizontal bar chart showing total FLC grouped by Job Function. Sum of all bars equals Total Labor Spend KPI.</t>
   </si>
   <si>
     <t>TC-008</t>
   </si>
   <si>
-    <t>Tabla de desglose geográfico</t>
-  </si>
-  <si>
-    <t>1. Localizar la tabla de desglose geográfico</t>
-  </si>
-  <si>
-    <t>Tabla con columnas: País, Headcount, % del Total, Labor Spend. Muestra hasta 10 países. El total de headcount suma correctamente al total general.</t>
+    <t>Geographic breakdown table</t>
+  </si>
+  <si>
+    <t>1. Locate the geographic breakdown table</t>
+  </si>
+  <si>
+    <t>Table with columns: Country, Headcount, % of Total, Labor Spend. Shows up to 10 countries. Headcount totals correctly to the overall total.</t>
   </si>
   <si>
     <t>TC-009</t>
   </si>
   <si>
-    <t>Flujo 2 — Datos Financieros</t>
-  </si>
-  <si>
-    <t>Obtener datos financieros por ticker (SEC EDGAR)</t>
-  </si>
-  <si>
-    <t>El usuario tiene el ticker de una empresa pública con 10-K presentado (ej. AAPL, MSFT)</t>
-  </si>
-  <si>
-    <t>1. Navegar a la pantalla de Datos Financieros
-2. Seleccionar modo Auto
-3. Ingresar el ticker
-4. Enviar la solicitud</t>
-  </si>
-  <si>
-    <t>El sistema consulta SEC EDGAR y devuelve: nombre de empresa, ticker, CIK, año fiscal, Revenue, EBITDA, Operating Income, D&amp;A, Total Expenses y desglose de gastos. Se muestra la fecha del filing y la fuente SEC EDGAR 10-K.</t>
+    <t>Flow 2 — Financial Data</t>
+  </si>
+  <si>
+    <t>Retrieve financial data by ticker (SEC EDGAR auto mode)</t>
+  </si>
+  <si>
+    <t>User has the ticker of a public company that has filed a 10-K (e.g. AAPL, MSFT)</t>
+  </si>
+  <si>
+    <t>1. Navigate to the Financial Data screen
+2. Select Auto mode
+3. Enter the ticker
+4. Submit the request</t>
+  </si>
+  <si>
+    <t>System queries SEC EDGAR and returns: company name, ticker, CIK, fiscal year, Revenue, EBITDA, Operating Income, D&amp;A, Total Expenses and expense breakdown (Cost of Revenue, R&amp;D, SG&amp;A). Filing date and source SEC EDGAR 10-K are shown.</t>
   </si>
   <si>
     <t>TC-010</t>
   </si>
   <si>
-    <t>Los datos corresponden al 10-K más reciente</t>
-  </si>
-  <si>
-    <t>TC-009 aprobado</t>
-  </si>
-  <si>
-    <t>1. Observar el campo de año fiscal y fecha de filing mostrados</t>
-  </si>
-  <si>
-    <t>Los datos corresponden al filing anual 10-K más reciente disponible en SEC EDGAR, no a un año anterior.</t>
+    <t>Financial data corresponds to the most recent 10-K</t>
+  </si>
+  <si>
+    <t>TC-009 passed</t>
+  </si>
+  <si>
+    <t>1. Observe the fiscal year and filing date shown</t>
+  </si>
+  <si>
+    <t>Data corresponds to the most recent annual 10-K filing available in SEC EDGAR, not a prior year.</t>
   </si>
   <si>
     <t>TC-011</t>
   </si>
   <si>
-    <t>Ingreso manual de datos financieros</t>
-  </si>
-  <si>
-    <t>El usuario tiene los datos financieros de la empresa disponibles</t>
-  </si>
-  <si>
-    <t>1. Seleccionar modo Manual
-2. Completar: Company Name, Fiscal Year, Total Revenue, EBITDA, Total Expenses
-3. (Opcional) Completar Cost of Revenue, R&amp;D, SG&amp;A
-4. Hacer clic en Save &amp; Apply</t>
-  </si>
-  <si>
-    <t>Los datos son aceptados y se muestran en pantalla. La fuente se indica como Manual Entry. El sistema acepta valores con formato de moneda (con $ y comas).</t>
+    <t>Manual financial data entry</t>
+  </si>
+  <si>
+    <t>User has the company's financial data available</t>
+  </si>
+  <si>
+    <t>1. Select Manual mode
+2. Fill in: Company Name, Fiscal Year, Total Revenue, EBITDA, Total Expenses
+3. (Optional) Fill in Cost of Revenue, R&amp;D, SG&amp;A
+4. Click Save &amp; Apply</t>
+  </si>
+  <si>
+    <t>Data is accepted and displayed on screen. Source is shown as Manual Entry. System accepts currency-formatted values (with $ and commas).</t>
   </si>
   <si>
     <t>TC-012</t>
   </si>
   <si>
-    <t>Flujo 3 — Análisis Integrado</t>
-  </si>
-  <si>
-    <t>Bloqueo de acceso sin ambas fuentes cargadas</t>
-  </si>
-  <si>
-    <t>Solo una de las dos fuentes está cargada (roster O financials)</t>
-  </si>
-  <si>
-    <t>1. Intentar navegar a la pantalla de Análisis Integrado</t>
-  </si>
-  <si>
-    <t>La pantalla muestra un indicador de bloqueo con checklist indicando qué fuente falta. No es posible acceder al análisis hasta tener ambas.</t>
+    <t>Flow 3 — Integrated Analysis</t>
+  </si>
+  <si>
+    <t>Navigation gate without both sources loaded</t>
+  </si>
+  <si>
+    <t>Only one source is loaded (roster OR financials, not both)</t>
+  </si>
+  <si>
+    <t>1. Attempt to navigate to the Integrated Analysis screen</t>
+  </si>
+  <si>
+    <t>Screen shows a lock indicator with a checklist indicating which source is missing. Access is not possible until both sources are loaded.</t>
   </si>
   <si>
     <t>TC-013</t>
   </si>
   <si>
-    <t>Modal de advertencia por desfase de período</t>
-  </si>
-  <si>
-    <t>Ambas fuentes cargadas. Primera vez que se accede al análisis integrado en la sesión.</t>
-  </si>
-  <si>
-    <t>1. Navegar a la pantalla de Análisis Integrado</t>
-  </si>
-  <si>
-    <t>Se muestra el modal Check your data periods advirtiendo al usuario que verifique que ambos datasets sean comparables temporalmente. El usuario puede cerrarlo y continuar.</t>
+    <t>Data period mismatch warning modal</t>
+  </si>
+  <si>
+    <t>Both sources loaded. First time accessing integrated analysis in the session.</t>
+  </si>
+  <si>
+    <t>1. Navigate to the Integrated Analysis screen</t>
+  </si>
+  <si>
+    <t>A modal Check your data periods is displayed, warning the user to verify both datasets cover comparable timeframes. User can dismiss it and continue.</t>
   </si>
   <si>
     <t>TC-014</t>
@@ -269,25 +269,25 @@
     <t>KPI: Revenue per Employee</t>
   </si>
   <si>
-    <t>TC-013 aprobado</t>
-  </si>
-  <si>
-    <t>1. Localizar la tarjeta de KPI Revenue per Employee</t>
-  </si>
-  <si>
-    <t>El valor mostrado es igual a Total Revenue (financials) / Total Headcount (roster). El resultado es matemáticamente correcto.</t>
+    <t>TC-013 passed</t>
+  </si>
+  <si>
+    <t>1. Locate the Revenue per Employee KPI card</t>
+  </si>
+  <si>
+    <t>Value displayed equals Total Revenue (financials) / Total Headcount (roster). Result is mathematically correct.</t>
   </si>
   <si>
     <t>TC-015</t>
   </si>
   <si>
-    <t>KPI: Labor Spend como % de Revenue</t>
-  </si>
-  <si>
-    <t>1. Localizar la tarjeta de KPI Labor Spend as % of Revenue</t>
-  </si>
-  <si>
-    <t>El valor es igual a Total Labor Spend / Total Revenue * 100. Si el resultado es menor al 1%, se muestra con decimales (no como 0%).</t>
+    <t>KPI: Labor Spend as % of Revenue</t>
+  </si>
+  <si>
+    <t>1. Locate the Labor Spend as % of Revenue KPI card</t>
+  </si>
+  <si>
+    <t>Value equals Total Labor Spend / Total Revenue * 100. If result is below 1%, it is shown with decimals (not as 0%).</t>
   </si>
   <si>
     <t>TC-016</t>
@@ -296,61 +296,61 @@
     <t>KPI: EBITDA Margin</t>
   </si>
   <si>
-    <t>1. Localizar la tarjeta de KPI EBITDA Margin</t>
-  </si>
-  <si>
-    <t>El valor es igual a EBITDA / Total Revenue * 100. El resultado es matemáticamente correcto.</t>
+    <t>1. Locate the EBITDA Margin KPI card</t>
+  </si>
+  <si>
+    <t>Value equals EBITDA / Total Revenue * 100. Result is mathematically correct.</t>
   </si>
   <si>
     <t>TC-017</t>
   </si>
   <si>
-    <t>Banner de comparación — resumen de ambas fuentes</t>
-  </si>
-  <si>
-    <t>1. Observar el banner superior de la pantalla de Análisis Integrado</t>
-  </si>
-  <si>
-    <t>El banner muestra a la izquierda datos del roster (nombre del archivo, headcount, países) y a la derecha datos financieros (empresa, año fiscal, revenue, EBITDA margin). El botón Export to PPT está visible y habilitado.</t>
+    <t>Comparison banner — summary of both sources</t>
+  </si>
+  <si>
+    <t>1. Observe the top banner on the Integrated Analysis screen</t>
+  </si>
+  <si>
+    <t>Banner shows on the left: roster data (file name, headcount, countries); on the right: financial data (company, fiscal year, revenue, EBITDA margin). Export to PPT button is visible and enabled.</t>
   </si>
   <si>
     <t>TC-018</t>
   </si>
   <si>
-    <t>Pirámide de seniority en análisis integrado</t>
-  </si>
-  <si>
-    <t>1. Localizar la visualización de pirámide de seniority</t>
-  </si>
-  <si>
-    <t>Gráfico de barras horizontales ordenado por jerarquía organizacional (niveles más senior arriba). La distribución es consistente con los datos del roster cargado.</t>
+    <t>Seniority pyramid in integrated analysis</t>
+  </si>
+  <si>
+    <t>1. Locate the seniority pyramid visualization</t>
+  </si>
+  <si>
+    <t>Horizontal bar chart ordered by org hierarchy (most senior at top). Distribution is consistent with the loaded roster data.</t>
   </si>
   <si>
     <t>TC-019</t>
   </si>
   <si>
-    <t>Oportunidades de valor: senior layer rationalization</t>
-  </si>
-  <si>
-    <t>TC-013 aprobado. VP + Director &gt; 20% del headcount total.</t>
-  </si>
-  <si>
-    <t>1. Localizar la sección Value Creation Opportunities</t>
-  </si>
-  <si>
-    <t>Se muestra la oportunidad Senior layer rationalization con el porcentaje actual de VP/Director y un impacto estimado calculado como reducción del 15% de ese grupo por su FLC promedio.</t>
+    <t>Value creation opportunity: senior layer rationalization</t>
+  </si>
+  <si>
+    <t>TC-013 passed. Roster has VP + Director &gt; 20% of total headcount.</t>
+  </si>
+  <si>
+    <t>1. Locate the Value Creation Opportunities section</t>
+  </si>
+  <si>
+    <t>Senior layer rationalization opportunity is shown with the current VP/Director percentage and an estimated impact calculated as a 15% reduction of that group multiplied by their average FLC.</t>
   </si>
   <si>
     <t>TC-020</t>
   </si>
   <si>
-    <t>Exportar análisis a PowerPoint</t>
-  </si>
-  <si>
-    <t>1. Hacer clic en el botón Export to PPT en el banner superior</t>
-  </si>
-  <si>
-    <t>Se genera y descarga un archivo .pptx con las slides del análisis integrado. El archivo se descarga correctamente en el navegador.</t>
+    <t>Export analysis to PowerPoint</t>
+  </si>
+  <si>
+    <t>1. Click the Export to PPT button in the top banner</t>
+  </si>
+  <si>
+    <t>A .pptx file is generated and downloaded with the integrated analysis slides. File downloads correctly in the browser.</t>
   </si>
 </sst>
 </file>
@@ -780,7 +780,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF6ACE86-34C7-4460-9596-CBB8EFDC2984}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4B28CA8-ADFB-4A94-95D7-6CEF507D96A2}">
   <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>

</xml_diff>